<commit_message>
Add GPS selective scheduler workflow
</commit_message>
<xml_diff>
--- a/data/input_clients_template.xlsx
+++ b/data/input_clients_template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="1" r:id="R956e61e340444c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="1" r:id="Re05d205155e244cb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,27 +221,24 @@
         <x:v>sales_rep</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>lat</x:v>
+        <x:v>gps</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>lon</x:v>
+        <x:v>visit_frequency</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>visit_frequency</x:v>
+        <x:v>fixed_weekday</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>fixed_weekday</x:v>
+        <x:v>forbidden_weekdays</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>forbidden_weekdays</x:v>
+        <x:v>preferred_weekdays</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>preferred_weekdays</x:v>
+        <x:v>cluster_manual</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>cluster_manual</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -255,20 +252,17 @@
       <x:c r="C2" s="4" t="str">
         <x:v>Rep A</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="n">
-        <x:v>42.6977</x:v>
+      <x:c r="D2" s="4" t="str">
+        <x:v>42.6977,23.3219</x:v>
       </x:c>
       <x:c r="E2" s="4" t="n">
-        <x:v>23.3219</x:v>
-      </x:c>
-      <x:c r="F2" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="F2" s="4" t="str"/>
       <x:c r="G2" s="4" t="str"/>
       <x:c r="H2" s="4" t="str"/>
       <x:c r="I2" s="4" t="str"/>
-      <x:c r="J2" s="4" t="str"/>
-      <x:c r="K2" s="4" t="str">
+      <x:c r="J2" s="4" t="str">
         <x:v>Optional notes</x:v>
       </x:c>
     </x:row>

</xml_diff>